<commit_message>
Updated using Indonesia specific data
</commit_message>
<xml_diff>
--- a/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
+++ b/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/land/PLANAbPiaSY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8EABB3-40FE-5144-817D-3C4CE99B98D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F16E712-EE45-DC41-B1E1-B54F7EFDB768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="99">
   <si>
     <t>PLANAbPiaSY Potential Land Area Newly Affected by Policy in a Single Year</t>
   </si>
@@ -660,7 +660,13 @@
       <sheetData sheetId="16"/>
       <sheetData sheetId="17"/>
       <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
+      <sheetData sheetId="19">
+        <row r="4">
+          <cell r="A4">
+            <v>3.6666666666666665</v>
+          </cell>
+        </row>
+      </sheetData>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3414,13 +3420,7 @@
         <f>J3*J4</f>
         <v>1606150</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="N5">
-        <f>N3/N4</f>
-        <v>0</v>
-      </c>
+      <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>

</xml_diff>

<commit_message>
Updated with Indonesia specific data
</commit_message>
<xml_diff>
--- a/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
+++ b/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/land/PLANAbPiaSY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DA043D-FCA6-2D4C-9C12-24A6DEA6E73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF033EB-207D-1E4D-AD87-DE79FF73337A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -627,14 +627,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3435,23 +3435,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="E1" s="30" t="s">
+      <c r="B1" s="33"/>
+      <c r="E1" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="31"/>
+      <c r="F1" s="33"/>
       <c r="G1" s="13"/>
-      <c r="I1" s="30" t="s">
+      <c r="I1" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="31"/>
-      <c r="M1" s="30" t="s">
+      <c r="J1" s="33"/>
+      <c r="M1" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="N1" s="31"/>
+      <c r="N1" s="33"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -3568,7 +3568,7 @@
       <c r="O6">
         <v>1.5</v>
       </c>
-      <c r="P6" s="33">
+      <c r="P6" s="31">
         <v>2</v>
       </c>
     </row>
@@ -3673,10 +3673,10 @@
       </c>
     </row>
     <row r="13" spans="1:16" ht="21" x14ac:dyDescent="0.25">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="31"/>
+      <c r="B13" s="33"/>
       <c r="E13" s="16" t="s">
         <v>73</v>
       </c>
@@ -3899,7 +3899,7 @@
         <f>C40*1000000</f>
         <v>54363183.923399992</v>
       </c>
-      <c r="E40" s="32">
+      <c r="E40" s="30">
         <v>1.7</v>
       </c>
       <c r="F40" s="20">
@@ -3918,6 +3918,10 @@
       <c r="C41">
         <f>N4*B41</f>
         <v>34.965411478005002</v>
+      </c>
+      <c r="D41" s="20">
+        <f>C41*1000000</f>
+        <v>34965411.478004999</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated land structure (alpha);merged PLAN file
</commit_message>
<xml_diff>
--- a/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
+++ b/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/land/PLANAbPiaSY/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tfranc03/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF033EB-207D-1E4D-AD87-DE79FF73337A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D658B9EC-9C84-8542-B3C2-F5EF64FA274F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="28300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Set Asides" sheetId="2" r:id="rId2"/>
     <sheet name="CO2 Sequestrated" sheetId="5" r:id="rId3"/>
     <sheet name="Potential land area" sheetId="3" r:id="rId4"/>
-    <sheet name="PLANAbPiaSY" sheetId="4" r:id="rId5"/>
+    <sheet name="Scratchpad" sheetId="6" r:id="rId5"/>
+    <sheet name="PLANAbPiaSY" sheetId="4" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <definedNames>
     <definedName name="acres_per_hectare">#REF!</definedName>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="131">
   <si>
     <t>PLANAbPiaSY Potential Land Area Newly Affected by Policy in a Single Year</t>
   </si>
@@ -410,6 +411,39 @@
   </si>
   <si>
     <t xml:space="preserve">60 t CO2 per ha </t>
+  </si>
+  <si>
+    <t>Sums of the PLANAbPiaSY tab (for new structure)</t>
+  </si>
+  <si>
+    <t>Implied from 31 July PLAN file</t>
+  </si>
+  <si>
+    <t>Acres (since summed)</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Emissions aren't significant; another way to say "avoid defo"?</t>
+  </si>
+  <si>
+    <t>griscom</t>
+  </si>
+  <si>
+    <t>Griscom for Rice (WRONG)</t>
+  </si>
+  <si>
+    <t>Griscom: Reforestation</t>
+  </si>
+  <si>
+    <t>Griscom: Natural forest management</t>
+  </si>
+  <si>
+    <t>Griscom: Peatland Restoration</t>
+  </si>
+  <si>
+    <t>Values from Potential Land Area calcs</t>
   </si>
 </sst>
 </file>
@@ -582,7 +616,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -631,10 +665,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -657,10 +699,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>101600</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>174625</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4048125" cy="4448175"/>
     <xdr:pic>
@@ -681,6 +723,10 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12534900" y="1393825"/>
+          <a:ext cx="4048125" cy="4448175"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -698,7 +744,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>2082800</xdr:colOff>
+      <xdr:colOff>190500</xdr:colOff>
       <xdr:row>62</xdr:row>
       <xdr:rowOff>178982</xdr:rowOff>
     </xdr:to>
@@ -731,6 +777,99 @@
         <a:xfrm>
           <a:off x="0" y="8851900"/>
           <a:ext cx="7772400" cy="3417482"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>482600</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>97459</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDB70F79-FCCD-4083-385D-7BF2BCDA119A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16408400" y="8331200"/>
+          <a:ext cx="7772400" cy="1951659"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>584200</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>596900</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>59032</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D2B5D95-026A-294D-5F67-9662CF4C2B74}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="584200" y="3022600"/>
+          <a:ext cx="7772400" cy="5634332"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3423,35 +3562,36 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.33203125" customWidth="1"/>
-    <col min="2" max="3" width="10.6640625" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="40.33203125" customWidth="1"/>
     <col min="6" max="8" width="10.6640625" customWidth="1"/>
     <col min="9" max="9" width="43.1640625" customWidth="1"/>
     <col min="10" max="12" width="10.6640625" customWidth="1"/>
     <col min="13" max="13" width="35.1640625" customWidth="1"/>
-    <col min="14" max="14" width="11.6640625" customWidth="1"/>
+    <col min="14" max="14" width="18.1640625" customWidth="1"/>
     <col min="15" max="26" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="E1" s="32" t="s">
+      <c r="B1" s="35"/>
+      <c r="E1" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="33"/>
+      <c r="F1" s="35"/>
       <c r="G1" s="13"/>
-      <c r="I1" s="32" t="s">
+      <c r="I1" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="33"/>
-      <c r="M1" s="32" t="s">
+      <c r="J1" s="35"/>
+      <c r="M1" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="N1" s="33"/>
+      <c r="N1" s="35"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -3507,6 +3647,9 @@
       <c r="B4" s="2">
         <v>212.02</v>
       </c>
+      <c r="C4" s="2" t="s">
+        <v>125</v>
+      </c>
       <c r="E4" s="2" t="s">
         <v>70</v>
       </c>
@@ -3642,7 +3785,7 @@
       <c r="M9" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="N9" s="15">
+      <c r="N9" s="33">
         <f>(N8/N2)*N4</f>
         <v>123956516.0925658</v>
       </c>
@@ -3673,10 +3816,10 @@
       </c>
     </row>
     <row r="13" spans="1:16" ht="21" x14ac:dyDescent="0.25">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="33"/>
+      <c r="B13" s="35"/>
       <c r="E13" s="16" t="s">
         <v>73</v>
       </c>
@@ -3758,6 +3901,9 @@
       <c r="B18" s="2">
         <v>21.56</v>
       </c>
+      <c r="C18" s="2" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
@@ -3918,10 +4064,6 @@
       <c r="C41">
         <f>N4*B41</f>
         <v>34.965411478005002</v>
-      </c>
-      <c r="D41" s="20">
-        <f>C41*1000000</f>
-        <v>34965411.478004999</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4934,6 +5076,116 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DA1CAE4-3810-2440-B0A3-9A0D32C200D9}">
+  <dimension ref="A4:D47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="45.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="37" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="32">
+        <f>SUM(PLANAbPiaSY!B2:AZ2)</f>
+        <v>51102000</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="32">
+        <f>SUM(PLANAbPiaSY!B3:AZ3)</f>
+        <v>1364952507.6174879</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="32">
+        <f>SUM(PLANAbPiaSY!B4:AZ4)</f>
+        <v>232492080.46237782</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="32">
+        <f>SUM(PLANAbPiaSY!B5:AZ5)</f>
+        <v>81913650</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="32">
+        <f>SUM(PLANAbPiaSY!B6:AZ6)</f>
+        <v>35615574.001849368</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="32">
+        <f>SUM(PLANAbPiaSY!B7:AZ7)</f>
+        <v>296138212.91485363</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B47" s="32"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FF1F497D"/>

</xml_diff>